<commit_message>
chore: corrige mensagem do commit
</commit_message>
<xml_diff>
--- a/teste-verzel-matriz-testes.xlsx
+++ b/teste-verzel-matriz-testes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADM\Documents\Programming\Verzel\Teste Técnico - Verzel Store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B225598-5146-4C6A-AA90-0F616F92CF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE4322F-6E35-40B1-A8CD-A0D7CFBA8851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos UI" sheetId="1" r:id="rId1"/>
@@ -4299,6 +4299,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-9B64-4D45-9A82-59A7977E97CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -4572,6 +4577,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-E2F4-4366-A3EE-C528234848A8}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -8130,7 +8140,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="10" t="s">
         <v>223</v>
       </c>
       <c r="B5">
@@ -8166,7 +8176,7 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="10" t="s">
         <v>227</v>
       </c>
       <c r="B9">
@@ -8175,6 +8185,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="BUGS!A2" display="UI — Falhou" xr:uid="{9BC09314-ED96-481A-8760-6B3D9F3440BC}"/>
+    <hyperlink ref="A9" location="BUGS!A3" display="API — Falhou" xr:uid="{0FB67E13-2BA2-4909-999C-275C82F4D85F}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
test(matriz): adiciona severidade e ajusta prioridades dos testes de API
</commit_message>
<xml_diff>
--- a/teste-verzel-matriz-testes.xlsx
+++ b/teste-verzel-matriz-testes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADM\Documents\Programming\Verzel\Teste Técnico - Verzel Store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE4322F-6E35-40B1-A8CD-A0D7CFBA8851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA38BD95-EF7A-4E98-ADC7-9185E9421A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos UI" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="358">
   <si>
     <t>ID</t>
   </si>
@@ -3060,70 +3060,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> retornar o resumo do cálculo.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Dado</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> um nome sem primeiro e último nome; 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Quando</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> criar o pedido; 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Então</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> rejeitar os dados e informar o campo inválido.</t>
     </r>
   </si>
   <si>
@@ -4083,6 +4019,97 @@
   </si>
   <si>
     <t>O esperado era que uma quantidade acima de 5 itens do mesmo produto não deveria ser aceita.</t>
+  </si>
+  <si>
+    <t>Severidade</t>
+  </si>
+  <si>
+    <t>Bloqueante</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dado</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> um nome sem primeiro e último nome; 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quando</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> criar o pedido; 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Então</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> rejeitar os dados; 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> informar o campo inválido.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4191,9 +4218,15 @@
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -5954,17 +5987,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CasosUI" displayName="CasosUI" ref="A1:I19">
-  <autoFilter ref="A1:I19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CasosUI" displayName="CasosUI" ref="A1:J19">
+  <autoFilter ref="A1:J19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Funcionalidade"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Cenário"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Requisito"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Prioridade"/>
+    <tableColumn id="10" xr3:uid="{51B02C10-CC2F-4CC8-8D23-46FBD80BE7B3}" name="Severidade" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="BDD"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evidências" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evidências" dataDxfId="1"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Bug"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -5972,14 +6006,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="CasosAPI" displayName="CasosAPI" ref="A1:L23">
-  <autoFilter ref="A1:L23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="CasosAPI" displayName="CasosAPI" ref="A1:M23">
+  <autoFilter ref="A1:M23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Funcionalidade"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Cenário"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Endpoint"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Prioridade"/>
+    <tableColumn id="13" xr3:uid="{DF090452-911D-4E92-AA62-05EDE4E5995C}" name="Severidade" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="BDD"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="HTTP Esperado"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Código Esperado"/>
@@ -6277,7 +6312,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6285,13 +6320,14 @@
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="78" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="28" style="8" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="78" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="28" style="8" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6307,20 +6343,23 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -6333,21 +6372,20 @@
       <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
@@ -6360,21 +6398,20 @@
       <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -6387,21 +6424,20 @@
       <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="I4" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -6414,21 +6450,20 @@
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="I5" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -6441,21 +6476,20 @@
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="I6" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
@@ -6468,21 +6502,20 @@
       <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
@@ -6495,21 +6528,20 @@
       <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="I8" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>33</v>
       </c>
@@ -6522,21 +6554,20 @@
       <c r="D9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="I9" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -6549,21 +6580,20 @@
       <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
@@ -6576,23 +6606,22 @@
       <c r="D11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="I11" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="J11" s="10" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -6605,21 +6634,20 @@
       <c r="D12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="I12" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -6632,21 +6660,20 @@
       <c r="D13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>48</v>
       </c>
@@ -6659,21 +6686,20 @@
       <c r="D14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="I14" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>52</v>
       </c>
@@ -6686,21 +6712,20 @@
       <c r="D15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="I15" s="2"/>
-    </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>55</v>
       </c>
@@ -6713,21 +6738,20 @@
       <c r="D16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="I16" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>59</v>
       </c>
@@ -6740,21 +6764,20 @@
       <c r="D17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
@@ -6767,21 +6790,20 @@
       <c r="D18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="I18" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>63</v>
       </c>
@@ -6794,46 +6816,45 @@
       <c r="D19" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="2" t="s">
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G19" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="H2:H19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Não executado,Passou,Falhou,Bloqueado,Não aplicável"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{38D03D3A-732C-494B-987A-77907072AFA8}"/>
-    <hyperlink ref="H12" r:id="rId2" xr:uid="{1B70BF68-0073-49DC-A574-0A4FC3D9FA83}"/>
-    <hyperlink ref="H11" r:id="rId3" xr:uid="{A627832B-AE3C-4BD1-B2F1-53C34228EDD6}"/>
-    <hyperlink ref="H10" r:id="rId4" xr:uid="{01A1674C-DC60-4469-A0EB-EF485C6FFA37}"/>
-    <hyperlink ref="H13" r:id="rId5" xr:uid="{A9279CEB-B83A-4EFD-AD8A-D6BE08F6CF2A}"/>
-    <hyperlink ref="H14" r:id="rId6" xr:uid="{0E452470-885C-478F-A01F-35BFACA36EFE}"/>
-    <hyperlink ref="H15" r:id="rId7" xr:uid="{645C0CE0-DFF7-43D3-91C5-9654CA7C9E29}"/>
-    <hyperlink ref="H18" r:id="rId8" xr:uid="{ADBEECF6-B6A5-404E-B163-6BECDF4AEBBF}"/>
-    <hyperlink ref="H17" r:id="rId9" xr:uid="{AF4D5327-467F-4F79-8AB8-8642FEE3329E}"/>
-    <hyperlink ref="H16" r:id="rId10" xr:uid="{D737B60B-CC63-4D75-BE93-ABA9FC646C6F}"/>
-    <hyperlink ref="H19" r:id="rId11" xr:uid="{D4C622CD-5ED1-42C7-96EB-4325AC0BED8C}"/>
-    <hyperlink ref="H6" r:id="rId12" xr:uid="{1E6F38C2-76D3-4425-8E90-3F2A195144F0}"/>
-    <hyperlink ref="H7" r:id="rId13" xr:uid="{188AA375-42F6-4394-8131-BBF2CAFF3C49}"/>
-    <hyperlink ref="H3" r:id="rId14" xr:uid="{34072715-4D6A-440D-9493-C0F88DC2EB15}"/>
-    <hyperlink ref="H4" r:id="rId15" xr:uid="{1DE85D6E-BBC3-4114-A8EC-4691142D9437}"/>
-    <hyperlink ref="H5" r:id="rId16" xr:uid="{738EC00C-364A-4164-B653-7036019DA312}"/>
-    <hyperlink ref="H8" r:id="rId17" xr:uid="{F16CCAF4-9BAB-48CD-9CFB-124354DA2314}"/>
-    <hyperlink ref="H9" r:id="rId18" xr:uid="{4E023B34-6EA8-4168-AC57-2FE592F00B4E}"/>
-    <hyperlink ref="I11" location="BUGS!A2" display="BUG-001" xr:uid="{9384DCDF-53AB-4FD6-BF12-5C544001807C}"/>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{38D03D3A-732C-494B-987A-77907072AFA8}"/>
+    <hyperlink ref="I12" r:id="rId2" xr:uid="{1B70BF68-0073-49DC-A574-0A4FC3D9FA83}"/>
+    <hyperlink ref="I11" r:id="rId3" xr:uid="{A627832B-AE3C-4BD1-B2F1-53C34228EDD6}"/>
+    <hyperlink ref="I10" r:id="rId4" xr:uid="{01A1674C-DC60-4469-A0EB-EF485C6FFA37}"/>
+    <hyperlink ref="I13" r:id="rId5" xr:uid="{A9279CEB-B83A-4EFD-AD8A-D6BE08F6CF2A}"/>
+    <hyperlink ref="I14" r:id="rId6" xr:uid="{0E452470-885C-478F-A01F-35BFACA36EFE}"/>
+    <hyperlink ref="I15" r:id="rId7" xr:uid="{645C0CE0-DFF7-43D3-91C5-9654CA7C9E29}"/>
+    <hyperlink ref="I18" r:id="rId8" xr:uid="{ADBEECF6-B6A5-404E-B163-6BECDF4AEBBF}"/>
+    <hyperlink ref="I17" r:id="rId9" xr:uid="{AF4D5327-467F-4F79-8AB8-8642FEE3329E}"/>
+    <hyperlink ref="I16" r:id="rId10" xr:uid="{D737B60B-CC63-4D75-BE93-ABA9FC646C6F}"/>
+    <hyperlink ref="I19" r:id="rId11" xr:uid="{D4C622CD-5ED1-42C7-96EB-4325AC0BED8C}"/>
+    <hyperlink ref="I6" r:id="rId12" xr:uid="{1E6F38C2-76D3-4425-8E90-3F2A195144F0}"/>
+    <hyperlink ref="I7" r:id="rId13" xr:uid="{188AA375-42F6-4394-8131-BBF2CAFF3C49}"/>
+    <hyperlink ref="I3" r:id="rId14" xr:uid="{34072715-4D6A-440D-9493-C0F88DC2EB15}"/>
+    <hyperlink ref="I4" r:id="rId15" xr:uid="{1DE85D6E-BBC3-4114-A8EC-4691142D9437}"/>
+    <hyperlink ref="I5" r:id="rId16" xr:uid="{738EC00C-364A-4164-B653-7036019DA312}"/>
+    <hyperlink ref="I8" r:id="rId17" xr:uid="{F16CCAF4-9BAB-48CD-9CFB-124354DA2314}"/>
+    <hyperlink ref="I9" r:id="rId18" xr:uid="{4E023B34-6EA8-4168-AC57-2FE592F00B4E}"/>
+    <hyperlink ref="J11" location="BUGS!A2" display="BUG-001" xr:uid="{9384DCDF-53AB-4FD6-BF12-5C544001807C}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
@@ -6845,24 +6866,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="76" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
-    <col min="9" max="9" width="72" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="32" customWidth="1"/>
+    <col min="10" max="10" width="72" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6878,29 +6900,32 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>71</v>
       </c>
@@ -6917,26 +6942,29 @@
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>322</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>75</v>
       </c>
@@ -6953,26 +6981,29 @@
         <v>12</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>322</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="L3" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M3" s="2"/>
+    </row>
+    <row r="4" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>78</v>
       </c>
@@ -6986,29 +7017,32 @@
         <v>77</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M4" s="2"/>
+    </row>
+    <row r="5" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>83</v>
       </c>
@@ -7025,26 +7059,29 @@
         <v>12</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="L5" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>90</v>
       </c>
@@ -7061,26 +7098,29 @@
         <v>12</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>93</v>
       </c>
@@ -7097,26 +7137,29 @@
         <v>12</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>97</v>
       </c>
@@ -7133,26 +7176,29 @@
         <v>12</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="L8" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M8" s="2"/>
+    </row>
+    <row r="9" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>100</v>
       </c>
@@ -7169,26 +7215,29 @@
         <v>12</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M9" s="2"/>
+    </row>
+    <row r="10" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>104</v>
       </c>
@@ -7205,26 +7254,29 @@
         <v>12</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="L10" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>108</v>
       </c>
@@ -7241,28 +7293,31 @@
         <v>42</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="M11" s="5" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>112</v>
       </c>
@@ -7279,26 +7334,29 @@
         <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>323</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="L12" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M12" s="2"/>
+    </row>
+    <row r="13" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>117</v>
       </c>
@@ -7312,29 +7370,32 @@
         <v>115</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>304</v>
+        <v>18</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="J13" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="L13" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>121</v>
       </c>
@@ -7348,29 +7409,32 @@
         <v>115</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>305</v>
-      </c>
       <c r="G14" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="J14" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K14" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="L14" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>122</v>
       </c>
@@ -7387,26 +7451,29 @@
         <v>12</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="G15" s="9">
+        <v>12</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="H15" s="9">
         <v>422</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="J15" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="L15" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>124</v>
       </c>
@@ -7420,29 +7487,32 @@
         <v>115</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>307</v>
-      </c>
       <c r="G16" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="I16" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="J16" s="2" t="s">
+      <c r="K16" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K16" s="5" t="s">
+      <c r="L16" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M16" s="2"/>
+    </row>
+    <row r="17" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>125</v>
       </c>
@@ -7456,29 +7526,32 @@
         <v>115</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>308</v>
-      </c>
       <c r="G17" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>323</v>
-      </c>
       <c r="I17" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="J17" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="L17" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="M17" s="2"/>
+    </row>
+    <row r="18" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>127</v>
       </c>
@@ -7495,26 +7568,29 @@
         <v>12</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>309</v>
+        <v>12</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K18" s="5" t="s">
+      <c r="L18" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M18" s="2"/>
+    </row>
+    <row r="19" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>129</v>
       </c>
@@ -7531,26 +7607,29 @@
         <v>12</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>310</v>
+        <v>12</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M19" s="2"/>
+    </row>
+    <row r="20" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>131</v>
       </c>
@@ -7567,26 +7646,29 @@
         <v>12</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>311</v>
+        <v>12</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="K20" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="L20" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>135</v>
       </c>
@@ -7603,26 +7685,29 @@
         <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>312</v>
+        <v>18</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="J21" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K21" s="5" t="s">
+      <c r="L21" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M21" s="2"/>
+    </row>
+    <row r="22" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>139</v>
       </c>
@@ -7639,26 +7724,29 @@
         <v>18</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>313</v>
+        <v>18</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="J22" s="2" t="s">
+      <c r="K22" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K22" s="5" t="s">
+      <c r="L22" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="M22" s="2"/>
+    </row>
+    <row r="23" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>146</v>
       </c>
@@ -7675,56 +7763,59 @@
         <v>18</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>314</v>
+        <v>18</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="I23" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="J23" s="2" t="s">
+      <c r="K23" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="K23" s="5" t="s">
+      <c r="L23" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="J2:J23" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" sqref="K2:K23" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Não executado,Passou,Falhou,Bloqueado,Não aplicável"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="K2" r:id="rId1" xr:uid="{D2957EEB-90F8-4CFE-B167-4DE666ECEEF6}"/>
-    <hyperlink ref="K3" r:id="rId2" xr:uid="{C4E8C425-97B1-49A2-B309-D3077E685DB7}"/>
-    <hyperlink ref="K4" r:id="rId3" xr:uid="{39E1966E-26AF-46FE-9E5E-7EF6D57B7341}"/>
-    <hyperlink ref="K5" r:id="rId4" xr:uid="{8BCD6219-EB16-475F-AAA5-A6227A1716E8}"/>
-    <hyperlink ref="K6" r:id="rId5" xr:uid="{01C37C90-43AE-416F-88FB-EBDA5802EE89}"/>
-    <hyperlink ref="K7" r:id="rId6" xr:uid="{16BADA19-BF87-4E18-B1F6-C443D41BF954}"/>
-    <hyperlink ref="K8" r:id="rId7" xr:uid="{2B9C1E15-826B-456E-8EED-6AE0AB8CB61A}"/>
-    <hyperlink ref="K9" r:id="rId8" xr:uid="{8F42F955-95DA-4DE7-B1F3-18CFAEB579D8}"/>
-    <hyperlink ref="K10" r:id="rId9" xr:uid="{DEE30BE1-0333-4494-9311-E38ED3A57A27}"/>
-    <hyperlink ref="K11" r:id="rId10" xr:uid="{94D0AF35-AF8B-43E8-92CC-D0FC6E379B4E}"/>
-    <hyperlink ref="K13" r:id="rId11" xr:uid="{DEA1F04B-A597-4CB0-8732-376EB64F93A1}"/>
-    <hyperlink ref="K12" r:id="rId12" xr:uid="{7279F4BF-8742-49C5-9EE0-853C840AFEF5}"/>
-    <hyperlink ref="K14" r:id="rId13" xr:uid="{9EE3D389-4256-4BB5-84DA-FAC5D5254630}"/>
-    <hyperlink ref="K15" r:id="rId14" xr:uid="{4687A703-1F91-497E-862D-1C0661205B26}"/>
-    <hyperlink ref="K16" r:id="rId15" xr:uid="{6432391A-BB05-47A3-84E6-88456B6FC901}"/>
-    <hyperlink ref="K17" r:id="rId16" xr:uid="{A581003B-B4DD-4BDE-8BFE-94CC693F42F4}"/>
-    <hyperlink ref="K18" r:id="rId17" xr:uid="{6EC1F558-88E2-4723-9493-D74E2863CD3A}"/>
-    <hyperlink ref="K19" r:id="rId18" xr:uid="{22C3ABE1-0585-40D8-893A-280C885F5872}"/>
-    <hyperlink ref="K20" r:id="rId19" xr:uid="{E8B249F2-FAD2-43F7-91CD-7821357898BD}"/>
-    <hyperlink ref="K21" r:id="rId20" xr:uid="{3EA84EC1-5520-47F1-88B6-1B6B9CC80F38}"/>
-    <hyperlink ref="K22" r:id="rId21" xr:uid="{45A5A0D8-CAF0-49BE-A206-C53106346C72}"/>
-    <hyperlink ref="K23" r:id="rId22" xr:uid="{4D492FF8-D268-46D1-A902-FC1192C6C18E}"/>
-    <hyperlink ref="L11" location="BUGS!A3" display="BUG-002" xr:uid="{291C3389-AB10-4D47-BB4D-B806062C4FA2}"/>
+    <hyperlink ref="L2" r:id="rId1" xr:uid="{D2957EEB-90F8-4CFE-B167-4DE666ECEEF6}"/>
+    <hyperlink ref="L3" r:id="rId2" xr:uid="{C4E8C425-97B1-49A2-B309-D3077E685DB7}"/>
+    <hyperlink ref="L4" r:id="rId3" xr:uid="{39E1966E-26AF-46FE-9E5E-7EF6D57B7341}"/>
+    <hyperlink ref="L5" r:id="rId4" xr:uid="{8BCD6219-EB16-475F-AAA5-A6227A1716E8}"/>
+    <hyperlink ref="L6" r:id="rId5" xr:uid="{01C37C90-43AE-416F-88FB-EBDA5802EE89}"/>
+    <hyperlink ref="L7" r:id="rId6" xr:uid="{16BADA19-BF87-4E18-B1F6-C443D41BF954}"/>
+    <hyperlink ref="L8" r:id="rId7" xr:uid="{2B9C1E15-826B-456E-8EED-6AE0AB8CB61A}"/>
+    <hyperlink ref="L9" r:id="rId8" xr:uid="{8F42F955-95DA-4DE7-B1F3-18CFAEB579D8}"/>
+    <hyperlink ref="L10" r:id="rId9" xr:uid="{DEE30BE1-0333-4494-9311-E38ED3A57A27}"/>
+    <hyperlink ref="L11" r:id="rId10" xr:uid="{94D0AF35-AF8B-43E8-92CC-D0FC6E379B4E}"/>
+    <hyperlink ref="L13" r:id="rId11" xr:uid="{DEA1F04B-A597-4CB0-8732-376EB64F93A1}"/>
+    <hyperlink ref="L12" r:id="rId12" xr:uid="{7279F4BF-8742-49C5-9EE0-853C840AFEF5}"/>
+    <hyperlink ref="L14" r:id="rId13" xr:uid="{9EE3D389-4256-4BB5-84DA-FAC5D5254630}"/>
+    <hyperlink ref="L15" r:id="rId14" xr:uid="{4687A703-1F91-497E-862D-1C0661205B26}"/>
+    <hyperlink ref="L16" r:id="rId15" xr:uid="{6432391A-BB05-47A3-84E6-88456B6FC901}"/>
+    <hyperlink ref="L17" r:id="rId16" xr:uid="{A581003B-B4DD-4BDE-8BFE-94CC693F42F4}"/>
+    <hyperlink ref="L18" r:id="rId17" xr:uid="{6EC1F558-88E2-4723-9493-D74E2863CD3A}"/>
+    <hyperlink ref="L19" r:id="rId18" xr:uid="{22C3ABE1-0585-40D8-893A-280C885F5872}"/>
+    <hyperlink ref="L20" r:id="rId19" xr:uid="{E8B249F2-FAD2-43F7-91CD-7821357898BD}"/>
+    <hyperlink ref="L21" r:id="rId20" xr:uid="{3EA84EC1-5520-47F1-88B6-1B6B9CC80F38}"/>
+    <hyperlink ref="L22" r:id="rId21" xr:uid="{45A5A0D8-CAF0-49BE-A206-C53106346C72}"/>
+    <hyperlink ref="L23" r:id="rId22" xr:uid="{4D492FF8-D268-46D1-A902-FC1192C6C18E}"/>
+    <hyperlink ref="M11" location="BUGS!A3" display="BUG-002" xr:uid="{291C3389-AB10-4D47-BB4D-B806062C4FA2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
@@ -7794,7 +7885,7 @@
         <v>166</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -7938,7 +8029,7 @@
         <v>197</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>198</v>
@@ -7955,7 +8046,7 @@
         <v>197</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>200</v>
@@ -7972,7 +8063,7 @@
         <v>197</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>202</v>
@@ -7981,7 +8072,7 @@
         <v>203</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -7989,7 +8080,7 @@
         <v>197</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>205</v>
@@ -8023,7 +8114,7 @@
         <v>197</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>207</v>
@@ -8040,7 +8131,7 @@
         <v>197</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>210</v>
@@ -8126,7 +8217,7 @@
         <v>221</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Casos UI'!G2:G19,"Não executado")</f>
+        <f>COUNTIF('Casos UI'!H2:H19,"Não executado")</f>
         <v>0</v>
       </c>
     </row>
@@ -8135,7 +8226,7 @@
         <v>222</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Casos UI'!G2:G19,"Passou")</f>
+        <f>COUNTIF('Casos UI'!H2:H19,"Passou")</f>
         <v>17</v>
       </c>
     </row>
@@ -8144,7 +8235,7 @@
         <v>223</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Casos UI'!G2:G19,"Falhou")</f>
+        <f>COUNTIF('Casos UI'!H2:H19,"Falhou")</f>
         <v>1</v>
       </c>
     </row>
@@ -8162,7 +8253,7 @@
         <v>225</v>
       </c>
       <c r="B7">
-        <f>COUNTIF('Casos API'!J2:J23,"Não executado")</f>
+        <f>COUNTIF('Casos API'!K2:K23,"Não executado")</f>
         <v>0</v>
       </c>
     </row>
@@ -8171,7 +8262,7 @@
         <v>226</v>
       </c>
       <c r="B8">
-        <f>COUNTIF('Casos API'!J2:J23,"Passou")</f>
+        <f>COUNTIF('Casos API'!K2:K23,"Passou")</f>
         <v>21</v>
       </c>
     </row>
@@ -8180,7 +8271,7 @@
         <v>227</v>
       </c>
       <c r="B9">
-        <f>COUNTIF('Casos API'!J2:J23,"Falhou")</f>
+        <f>COUNTIF('Casos API'!K2:K23,"Falhou")</f>
         <v>1</v>
       </c>
     </row>
@@ -8336,7 +8427,7 @@
         <v>115</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -8344,7 +8435,7 @@
         <v>142</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -8368,71 +8459,71 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B1" t="s">
         <v>336</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>337</v>
-      </c>
-      <c r="C1" t="s">
-        <v>338</v>
       </c>
       <c r="D1" t="s">
         <v>237</v>
       </c>
       <c r="E1" t="s">
+        <v>338</v>
+      </c>
+      <c r="F1" t="s">
         <v>339</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>340</v>
-      </c>
-      <c r="G1" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="207" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="E2" t="s">
         <v>343</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>347</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>344</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>345</v>
-      </c>
-      <c r="G2" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="180" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>348</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" t="s">
         <v>352</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" t="s">
         <v>354</v>
-      </c>
-      <c r="G3" t="s">
-        <v>355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(matriz): ajusta bug reports e casos de teste
</commit_message>
<xml_diff>
--- a/teste-verzel-matriz-testes.xlsx
+++ b/teste-verzel-matriz-testes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADM\Documents\Programming\Verzel\Teste Técnico - Verzel Store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA38BD95-EF7A-4E98-ADC7-9185E9421A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3F30DC-67AA-4304-B1E7-E0A1ADDCE1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Dados de Teste" sheetId="3" r:id="rId3"/>
     <sheet name="Resumo" sheetId="4" r:id="rId4"/>
     <sheet name="Rastreabilidade" sheetId="5" r:id="rId5"/>
-    <sheet name="BUGS" sheetId="6" r:id="rId6"/>
+    <sheet name="BUG REPORT" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados de Teste'!$A$1:$E$20</definedName>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="397">
   <si>
     <t>ID</t>
   </si>
@@ -254,9 +254,6 @@
     <t>Código Esperado</t>
   </si>
   <si>
-    <t>Quando acontece</t>
-  </si>
-  <si>
     <t>API-001</t>
   </si>
   <si>
@@ -3839,12 +3836,6 @@
   </si>
   <si>
     <t>Quando um CEP com 8 dígitos com hífen é informado.</t>
-  </si>
-  <si>
-    <t>Quando a requisição é aceita e os produtos disponíveis são mostradas corretamente.</t>
-  </si>
-  <si>
-    <t>Quando a requisição é aceita e as informações dos produtos disponíveis são mostradas corretamente.</t>
   </si>
   <si>
     <r>
@@ -3988,9 +3979,6 @@
     <t>URL: https://verzel-store.qa-test-verzel-store.workers.dev/</t>
   </si>
   <si>
-    <t>O esperado era que ao adicionar itens no carrinho de forma a atingir um subtotal de R$200,00 o valor do frete passasse a ser R$0,00.</t>
-  </si>
-  <si>
     <t>https://app.screencast.com/raVXqM0FR2aft</t>
   </si>
   <si>
@@ -4018,9 +4006,6 @@
     <t>URL: https://verzel-store.qa-test-verzel-store.workers.dev/api/carrinho/calcular</t>
   </si>
   <si>
-    <t>O esperado era que uma quantidade acima de 5 itens do mesmo produto não deveria ser aceita.</t>
-  </si>
-  <si>
     <t>Severidade</t>
   </si>
   <si>
@@ -4110,13 +4095,180 @@
       </rPr>
       <t xml:space="preserve"> informar o campo inválido.</t>
     </r>
+  </si>
+  <si>
+    <t>Resultado Obtido</t>
+  </si>
+  <si>
+    <t>Um desconto de 10% deve ser aplicado ao subtotal.</t>
+  </si>
+  <si>
+    <t>Não deve ser aplicado desconto.</t>
+  </si>
+  <si>
+    <t>A aplicação de multiplos cupons não deve ser aceita.</t>
+  </si>
+  <si>
+    <t>Segundo cupom deve ser aceito caso seja válido.</t>
+  </si>
+  <si>
+    <t>O valor do frete deve ser cobrado.</t>
+  </si>
+  <si>
+    <t>O frete deve ser grátis.</t>
+  </si>
+  <si>
+    <t>A mensagem com o correto valor faltante para frete grátis deve aparecer.</t>
+  </si>
+  <si>
+    <t>O frete grátis deve ser mantido.</t>
+  </si>
+  <si>
+    <t>Valor do frete deve ser mantido.</t>
+  </si>
+  <si>
+    <t>Quantidade selecionada deve ser aceita.</t>
+  </si>
+  <si>
+    <t>Quantidade requisitada não deve ser aceita.</t>
+  </si>
+  <si>
+    <t>Os valores mostrados devem possuir 2 casas decimais.</t>
+  </si>
+  <si>
+    <t>Conforme esperado.</t>
+  </si>
+  <si>
+    <t>O frete grátis não foi concedido.</t>
+  </si>
+  <si>
+    <t>O valor do frete deve ser R$ 0,00 (Frete Grátis).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A API deve retornar </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF303030"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>HTTP 400 Bad Request</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF303030"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t xml:space="preserve"> com o código de erro </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>QUANTIDADE_MAXIMA_EXCEDIDA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF303030"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>O sistema exibe "Faltam R$ 0,00 para o frete grátis", porém mantém o frete cobrado em R$ 19,90.</t>
+  </si>
+  <si>
+    <t>A API retorna HTTP 200 OK aceitando as 10 unidades e calculando o subtotal normalmente.</t>
+  </si>
+  <si>
+    <t>Pré-condições / Dados de entrada</t>
+  </si>
+  <si>
+    <t>Quando a requisição é aceita e os produtos disponíveis são mostrados corretamente.</t>
+  </si>
+  <si>
+    <t>Quando a requisição é aceita e as informações dos produtos disponíveis são mostrados corretamente.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 200 OK e uma lista com os produtos disponíveis, contendo os dados previstos no contrato da API.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 200 OK e os dados do produto correspondente ao ID informado.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 404 com o código PRODUTO_NAO_ENCONTRADO e a mensagem de erro correspondente.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código ITENS_OBRIGATORIOS e a mensagem informando a ausência do campo itens.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código ITENS_OBRIGATORIOS e a mensagem informando que o campo itens não pode estar vazio.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código ITEM_INVALIDO e a mensagem indicando a estrutura inválida do item ou a ausência de campos obrigatórios.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código PRODUTO_NAO_ENCONTRADO e a mensagem informando que o produto solicitado não existe.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código ITEM_DUPLICADO e a mensagem informando a duplicidade do produto na lista de itens.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código QUANTIDADE_INVALIDA e a mensagem indicando que a quantidade deve ser um inteiro maior ou igual a 1.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código QUANTIDADE_MAXIMA_EXCEDIDA e a mensagem informando que a quantidade máxima permitida é 5 unidades por produto.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 201 Created, o número do pedido no formato VZ-000000 e o resumo do cálculo, incluindo os valores correspondentes ao pedido criado.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código DADOS_INVALIDOS e indicar o campo de nome inválido por meio da mensagem ou dos detalhes de validação.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código DADOS_INVALIDOS e indicar que o e-mail informado possui formato inválido.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código DADOS_INVALIDOS e indicar que o campo nome é obrigatório.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 201 Created e criar o pedido aceitando o CEP com 8 dígitos sem hífen.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 201 Created e criar o pedido aceitando o CEP no formato 12345-678.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código DADOS_INVALIDOS e indicar que o CEP informado possui formato ou quantidade de dígitos inválidos.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código CUPOM_INVALIDO e a mensagem informando que o cupom não existe ou não é válido.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 422 com o código CUPOM_EXPIRADO e a mensagem informando que o cupom está expirado.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 405 com o código METODO_NAO_PERMITIDO e a mensagem correspondente ao método HTTP não permitido.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 404 com o código ROTA_NAO_ENCONTRADA e a mensagem informando que a rota solicitada não existe.</t>
+  </si>
+  <si>
+    <t>Retornar HTTP 400 com o código JSON_INVALIDO e a mensagem informando que o corpo da requisição contém JSON inválido.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4157,6 +4309,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF303030"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -4218,12 +4381,24 @@
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -5987,18 +6162,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CasosUI" displayName="CasosUI" ref="A1:J19">
-  <autoFilter ref="A1:J19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CasosUI" displayName="CasosUI" ref="A1:L19">
+  <autoFilter ref="A1:L19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Funcionalidade"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Cenário"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Requisito"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Prioridade"/>
-    <tableColumn id="10" xr3:uid="{51B02C10-CC2F-4CC8-8D23-46FBD80BE7B3}" name="Severidade" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{51B02C10-CC2F-4CC8-8D23-46FBD80BE7B3}" name="Severidade" dataDxfId="6"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="BDD"/>
+    <tableColumn id="11" xr3:uid="{0A888607-2E5E-4B78-B474-0292E91CA5A8}" name="Resultado Esperado" dataDxfId="5"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Status"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evidências" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{A78DE500-E00B-46DD-9772-C68FE2F9BC85}" name="Resultado Obtido" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evidências" dataDxfId="3"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Bug"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6006,20 +6183,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="CasosAPI" displayName="CasosAPI" ref="A1:M23">
-  <autoFilter ref="A1:M23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="CasosAPI" displayName="CasosAPI" ref="A1:O23">
+  <autoFilter ref="A1:O23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Funcionalidade"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Cenário"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Endpoint"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Prioridade"/>
-    <tableColumn id="13" xr3:uid="{DF090452-911D-4E92-AA62-05EDE4E5995C}" name="Severidade" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{DF090452-911D-4E92-AA62-05EDE4E5995C}" name="Severidade" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="BDD"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="HTTP Esperado"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Código Esperado"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Quando acontece"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Pré-condições / Dados de entrada"/>
+    <tableColumn id="14" xr3:uid="{87BD1CDD-4B5B-4C6B-8ABA-3AC215AE50F5}" name="Resultado Esperado" dataDxfId="1"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Status"/>
+    <tableColumn id="15" xr3:uid="{709BCEA5-F542-47A5-86EE-D0F0D031F682}" name="Resultado Obtido" dataDxfId="0"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Evidência"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Bug"/>
   </tableColumns>
@@ -6312,27 +6491,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="78" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="28" style="8" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="7" max="8" width="78" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28" style="8" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
@@ -6344,22 +6524,28 @@
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -6372,25 +6558,35 @@
       <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G2" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -6398,20 +6594,30 @@
       <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G3" s="2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -6424,20 +6630,30 @@
       <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -6450,20 +6666,30 @@
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G5" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -6476,20 +6702,30 @@
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G6" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
@@ -6502,20 +6738,30 @@
       <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G7" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
@@ -6528,20 +6774,30 @@
       <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G8" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>33</v>
       </c>
@@ -6554,20 +6810,30 @@
       <c r="D9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G9" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -6580,20 +6846,30 @@
       <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="E10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G10" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
@@ -6606,22 +6882,32 @@
       <c r="D11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="E11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G11" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H11" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="I11" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -6634,20 +6920,30 @@
       <c r="D12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="E12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G12" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -6660,20 +6956,30 @@
       <c r="D13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G13" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>48</v>
       </c>
@@ -6686,20 +6992,30 @@
       <c r="D14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G14" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>52</v>
       </c>
@@ -6712,20 +7028,30 @@
       <c r="D15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G15" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>362</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>55</v>
       </c>
@@ -6738,20 +7064,30 @@
       <c r="D16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G16" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>59</v>
       </c>
@@ -6764,20 +7100,30 @@
       <c r="D17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G17" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
@@ -6790,20 +7136,30 @@
       <c r="D18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="E18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="G18" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="J18" s="2"/>
-    </row>
-    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>364</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>63</v>
       </c>
@@ -6816,45 +7172,55 @@
       <c r="D19" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G19" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="J19" s="2"/>
+        <v>365</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="L19" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="H2:H19" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="I2:J19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Não executado,Passou,Falhou,Bloqueado,Não aplicável"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{38D03D3A-732C-494B-987A-77907072AFA8}"/>
-    <hyperlink ref="I12" r:id="rId2" xr:uid="{1B70BF68-0073-49DC-A574-0A4FC3D9FA83}"/>
-    <hyperlink ref="I11" r:id="rId3" xr:uid="{A627832B-AE3C-4BD1-B2F1-53C34228EDD6}"/>
-    <hyperlink ref="I10" r:id="rId4" xr:uid="{01A1674C-DC60-4469-A0EB-EF485C6FFA37}"/>
-    <hyperlink ref="I13" r:id="rId5" xr:uid="{A9279CEB-B83A-4EFD-AD8A-D6BE08F6CF2A}"/>
-    <hyperlink ref="I14" r:id="rId6" xr:uid="{0E452470-885C-478F-A01F-35BFACA36EFE}"/>
-    <hyperlink ref="I15" r:id="rId7" xr:uid="{645C0CE0-DFF7-43D3-91C5-9654CA7C9E29}"/>
-    <hyperlink ref="I18" r:id="rId8" xr:uid="{ADBEECF6-B6A5-404E-B163-6BECDF4AEBBF}"/>
-    <hyperlink ref="I17" r:id="rId9" xr:uid="{AF4D5327-467F-4F79-8AB8-8642FEE3329E}"/>
-    <hyperlink ref="I16" r:id="rId10" xr:uid="{D737B60B-CC63-4D75-BE93-ABA9FC646C6F}"/>
-    <hyperlink ref="I19" r:id="rId11" xr:uid="{D4C622CD-5ED1-42C7-96EB-4325AC0BED8C}"/>
-    <hyperlink ref="I6" r:id="rId12" xr:uid="{1E6F38C2-76D3-4425-8E90-3F2A195144F0}"/>
-    <hyperlink ref="I7" r:id="rId13" xr:uid="{188AA375-42F6-4394-8131-BBF2CAFF3C49}"/>
-    <hyperlink ref="I3" r:id="rId14" xr:uid="{34072715-4D6A-440D-9493-C0F88DC2EB15}"/>
-    <hyperlink ref="I4" r:id="rId15" xr:uid="{1DE85D6E-BBC3-4114-A8EC-4691142D9437}"/>
-    <hyperlink ref="I5" r:id="rId16" xr:uid="{738EC00C-364A-4164-B653-7036019DA312}"/>
-    <hyperlink ref="I8" r:id="rId17" xr:uid="{F16CCAF4-9BAB-48CD-9CFB-124354DA2314}"/>
-    <hyperlink ref="I9" r:id="rId18" xr:uid="{4E023B34-6EA8-4168-AC57-2FE592F00B4E}"/>
-    <hyperlink ref="J11" location="BUGS!A2" display="BUG-001" xr:uid="{9384DCDF-53AB-4FD6-BF12-5C544001807C}"/>
+    <hyperlink ref="K2" r:id="rId1" xr:uid="{38D03D3A-732C-494B-987A-77907072AFA8}"/>
+    <hyperlink ref="K12" r:id="rId2" xr:uid="{1B70BF68-0073-49DC-A574-0A4FC3D9FA83}"/>
+    <hyperlink ref="K11" r:id="rId3" xr:uid="{A627832B-AE3C-4BD1-B2F1-53C34228EDD6}"/>
+    <hyperlink ref="K10" r:id="rId4" xr:uid="{01A1674C-DC60-4469-A0EB-EF485C6FFA37}"/>
+    <hyperlink ref="K13" r:id="rId5" xr:uid="{A9279CEB-B83A-4EFD-AD8A-D6BE08F6CF2A}"/>
+    <hyperlink ref="K14" r:id="rId6" xr:uid="{0E452470-885C-478F-A01F-35BFACA36EFE}"/>
+    <hyperlink ref="K15" r:id="rId7" xr:uid="{645C0CE0-DFF7-43D3-91C5-9654CA7C9E29}"/>
+    <hyperlink ref="K18" r:id="rId8" xr:uid="{ADBEECF6-B6A5-404E-B163-6BECDF4AEBBF}"/>
+    <hyperlink ref="K17" r:id="rId9" xr:uid="{AF4D5327-467F-4F79-8AB8-8642FEE3329E}"/>
+    <hyperlink ref="K16" r:id="rId10" xr:uid="{D737B60B-CC63-4D75-BE93-ABA9FC646C6F}"/>
+    <hyperlink ref="K19" r:id="rId11" xr:uid="{D4C622CD-5ED1-42C7-96EB-4325AC0BED8C}"/>
+    <hyperlink ref="K6" r:id="rId12" xr:uid="{1E6F38C2-76D3-4425-8E90-3F2A195144F0}"/>
+    <hyperlink ref="K7" r:id="rId13" xr:uid="{188AA375-42F6-4394-8131-BBF2CAFF3C49}"/>
+    <hyperlink ref="K3" r:id="rId14" xr:uid="{34072715-4D6A-440D-9493-C0F88DC2EB15}"/>
+    <hyperlink ref="K4" r:id="rId15" xr:uid="{1DE85D6E-BBC3-4114-A8EC-4691142D9437}"/>
+    <hyperlink ref="K5" r:id="rId16" xr:uid="{738EC00C-364A-4164-B653-7036019DA312}"/>
+    <hyperlink ref="K8" r:id="rId17" xr:uid="{F16CCAF4-9BAB-48CD-9CFB-124354DA2314}"/>
+    <hyperlink ref="K9" r:id="rId18" xr:uid="{4E023B34-6EA8-4168-AC57-2FE592F00B4E}"/>
+    <hyperlink ref="L11" location="'BUG REPORT'!A2" display="BUG-001" xr:uid="{9384DCDF-53AB-4FD6-BF12-5C544001807C}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
@@ -6866,7 +7232,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6879,17 +7245,19 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="32" customWidth="1"/>
     <col min="10" max="10" width="72" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="11" max="11" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
@@ -6901,7 +7269,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -6913,69 +7281,81 @@
         <v>69</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="M2" s="2"/>
-    </row>
-    <row r="3" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
@@ -6984,37 +7364,43 @@
         <v>12</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>326</v>
+        <v>374</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="M3" s="2"/>
-    </row>
-    <row r="4" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>18</v>
@@ -7023,37 +7409,43 @@
         <v>18</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>12</v>
@@ -7062,37 +7454,43 @@
         <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="M5" s="2"/>
-    </row>
-    <row r="6" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>12</v>
@@ -7101,37 +7499,43 @@
         <v>12</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="J6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="M6" s="2"/>
-    </row>
-    <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
@@ -7140,37 +7544,43 @@
         <v>12</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="M7" s="2"/>
-    </row>
-    <row r="8" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>12</v>
@@ -7179,37 +7589,43 @@
         <v>12</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="M8" s="2"/>
-    </row>
-    <row r="9" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>12</v>
@@ -7218,37 +7634,43 @@
         <v>12</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="M9" s="2"/>
-    </row>
-    <row r="10" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>12</v>
@@ -7257,37 +7679,43 @@
         <v>12</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="M10" s="2"/>
-    </row>
-    <row r="11" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>42</v>
@@ -7296,78 +7724,90 @@
         <v>12</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>18</v>
@@ -7376,37 +7816,43 @@
         <v>18</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="M13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>42</v>
@@ -7415,37 +7861,43 @@
         <v>12</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L14" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N14" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>263</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>12</v>
@@ -7454,37 +7906,43 @@
         <v>12</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H15" s="9">
         <v>422</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="M15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>42</v>
@@ -7493,37 +7951,43 @@
         <v>12</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>323</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>42</v>
@@ -7532,37 +7996,43 @@
         <v>12</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L17" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="M17" s="2"/>
-    </row>
-    <row r="18" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>12</v>
@@ -7571,37 +8041,43 @@
         <v>12</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I18" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>120</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>12</v>
@@ -7610,37 +8086,43 @@
         <v>12</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I19" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="K19" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="M19" s="2"/>
-    </row>
-    <row r="20" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+        <v>392</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>12</v>
@@ -7649,37 +8131,43 @@
         <v>12</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I20" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="J20" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="K20" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L20" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="M20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+        <v>393</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N20" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="21" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>18</v>
@@ -7688,37 +8176,43 @@
         <v>18</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H21" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N21" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="O21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>140</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>18</v>
@@ -7727,37 +8221,43 @@
         <v>18</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J22" s="2" t="s">
+      <c r="K22" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N22" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>18</v>
@@ -7766,56 +8266,62 @@
         <v>18</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H23" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="K23" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="L23" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="M23" s="2"/>
+        <v>396</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N23" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="O23" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" sqref="K2:K23" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="L2:M23" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Não executado,Passou,Falhou,Bloqueado,Não aplicável"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="L2" r:id="rId1" xr:uid="{D2957EEB-90F8-4CFE-B167-4DE666ECEEF6}"/>
-    <hyperlink ref="L3" r:id="rId2" xr:uid="{C4E8C425-97B1-49A2-B309-D3077E685DB7}"/>
-    <hyperlink ref="L4" r:id="rId3" xr:uid="{39E1966E-26AF-46FE-9E5E-7EF6D57B7341}"/>
-    <hyperlink ref="L5" r:id="rId4" xr:uid="{8BCD6219-EB16-475F-AAA5-A6227A1716E8}"/>
-    <hyperlink ref="L6" r:id="rId5" xr:uid="{01C37C90-43AE-416F-88FB-EBDA5802EE89}"/>
-    <hyperlink ref="L7" r:id="rId6" xr:uid="{16BADA19-BF87-4E18-B1F6-C443D41BF954}"/>
-    <hyperlink ref="L8" r:id="rId7" xr:uid="{2B9C1E15-826B-456E-8EED-6AE0AB8CB61A}"/>
-    <hyperlink ref="L9" r:id="rId8" xr:uid="{8F42F955-95DA-4DE7-B1F3-18CFAEB579D8}"/>
-    <hyperlink ref="L10" r:id="rId9" xr:uid="{DEE30BE1-0333-4494-9311-E38ED3A57A27}"/>
-    <hyperlink ref="L11" r:id="rId10" xr:uid="{94D0AF35-AF8B-43E8-92CC-D0FC6E379B4E}"/>
-    <hyperlink ref="L13" r:id="rId11" xr:uid="{DEA1F04B-A597-4CB0-8732-376EB64F93A1}"/>
-    <hyperlink ref="L12" r:id="rId12" xr:uid="{7279F4BF-8742-49C5-9EE0-853C840AFEF5}"/>
-    <hyperlink ref="L14" r:id="rId13" xr:uid="{9EE3D389-4256-4BB5-84DA-FAC5D5254630}"/>
-    <hyperlink ref="L15" r:id="rId14" xr:uid="{4687A703-1F91-497E-862D-1C0661205B26}"/>
-    <hyperlink ref="L16" r:id="rId15" xr:uid="{6432391A-BB05-47A3-84E6-88456B6FC901}"/>
-    <hyperlink ref="L17" r:id="rId16" xr:uid="{A581003B-B4DD-4BDE-8BFE-94CC693F42F4}"/>
-    <hyperlink ref="L18" r:id="rId17" xr:uid="{6EC1F558-88E2-4723-9493-D74E2863CD3A}"/>
-    <hyperlink ref="L19" r:id="rId18" xr:uid="{22C3ABE1-0585-40D8-893A-280C885F5872}"/>
-    <hyperlink ref="L20" r:id="rId19" xr:uid="{E8B249F2-FAD2-43F7-91CD-7821357898BD}"/>
-    <hyperlink ref="L21" r:id="rId20" xr:uid="{3EA84EC1-5520-47F1-88B6-1B6B9CC80F38}"/>
-    <hyperlink ref="L22" r:id="rId21" xr:uid="{45A5A0D8-CAF0-49BE-A206-C53106346C72}"/>
-    <hyperlink ref="L23" r:id="rId22" xr:uid="{4D492FF8-D268-46D1-A902-FC1192C6C18E}"/>
-    <hyperlink ref="M11" location="BUGS!A3" display="BUG-002" xr:uid="{291C3389-AB10-4D47-BB4D-B806062C4FA2}"/>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{D2957EEB-90F8-4CFE-B167-4DE666ECEEF6}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{C4E8C425-97B1-49A2-B309-D3077E685DB7}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{39E1966E-26AF-46FE-9E5E-7EF6D57B7341}"/>
+    <hyperlink ref="N5" r:id="rId4" xr:uid="{8BCD6219-EB16-475F-AAA5-A6227A1716E8}"/>
+    <hyperlink ref="N6" r:id="rId5" xr:uid="{01C37C90-43AE-416F-88FB-EBDA5802EE89}"/>
+    <hyperlink ref="N7" r:id="rId6" xr:uid="{16BADA19-BF87-4E18-B1F6-C443D41BF954}"/>
+    <hyperlink ref="N8" r:id="rId7" xr:uid="{2B9C1E15-826B-456E-8EED-6AE0AB8CB61A}"/>
+    <hyperlink ref="N9" r:id="rId8" xr:uid="{8F42F955-95DA-4DE7-B1F3-18CFAEB579D8}"/>
+    <hyperlink ref="N10" r:id="rId9" xr:uid="{DEE30BE1-0333-4494-9311-E38ED3A57A27}"/>
+    <hyperlink ref="N11" r:id="rId10" xr:uid="{94D0AF35-AF8B-43E8-92CC-D0FC6E379B4E}"/>
+    <hyperlink ref="N13" r:id="rId11" xr:uid="{DEA1F04B-A597-4CB0-8732-376EB64F93A1}"/>
+    <hyperlink ref="N12" r:id="rId12" xr:uid="{7279F4BF-8742-49C5-9EE0-853C840AFEF5}"/>
+    <hyperlink ref="N14" r:id="rId13" xr:uid="{9EE3D389-4256-4BB5-84DA-FAC5D5254630}"/>
+    <hyperlink ref="N15" r:id="rId14" xr:uid="{4687A703-1F91-497E-862D-1C0661205B26}"/>
+    <hyperlink ref="N16" r:id="rId15" xr:uid="{6432391A-BB05-47A3-84E6-88456B6FC901}"/>
+    <hyperlink ref="N17" r:id="rId16" xr:uid="{A581003B-B4DD-4BDE-8BFE-94CC693F42F4}"/>
+    <hyperlink ref="N18" r:id="rId17" xr:uid="{6EC1F558-88E2-4723-9493-D74E2863CD3A}"/>
+    <hyperlink ref="N19" r:id="rId18" xr:uid="{22C3ABE1-0585-40D8-893A-280C885F5872}"/>
+    <hyperlink ref="N20" r:id="rId19" xr:uid="{E8B249F2-FAD2-43F7-91CD-7821357898BD}"/>
+    <hyperlink ref="N21" r:id="rId20" xr:uid="{3EA84EC1-5520-47F1-88B6-1B6B9CC80F38}"/>
+    <hyperlink ref="N22" r:id="rId21" xr:uid="{45A5A0D8-CAF0-49BE-A206-C53106346C72}"/>
+    <hyperlink ref="N23" r:id="rId22" xr:uid="{4D492FF8-D268-46D1-A902-FC1192C6C18E}"/>
+    <hyperlink ref="O11" location="'BUG REPORT'!A3" display="BUG-002" xr:uid="{291C3389-AB10-4D47-BB4D-B806062C4FA2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
@@ -7839,118 +8345,118 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>157</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>166</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>43</v>
@@ -7958,223 +8464,223 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>184</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>191</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>203</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>206</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B16" s="9">
         <v>12345678</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>211</v>
-      </c>
       <c r="E18" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="E20" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -8197,15 +8703,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B2">
         <f>COUNTA('Casos UI'!A2:A19)</f>
@@ -8214,34 +8720,34 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Casos UI'!H2:H19,"Não executado")</f>
+        <f>COUNTIF('Casos UI'!I2:I19,"Não executado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Casos UI'!H2:H19,"Passou")</f>
+        <f>COUNTIF('Casos UI'!I2:I19,"Passou")</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Casos UI'!H2:H19,"Falhou")</f>
+        <f>COUNTIF('Casos UI'!I2:I19,"Falhou")</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B6">
         <f>COUNTA('Casos API'!A2:A23)</f>
@@ -8250,35 +8756,35 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B7">
-        <f>COUNTIF('Casos API'!K2:K23,"Não executado")</f>
+        <f>COUNTIF('Casos API'!L2:L23,"Não executado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B8">
-        <f>COUNTIF('Casos API'!K2:K23,"Passou")</f>
+        <f>COUNTIF('Casos API'!L2:L23,"Passou")</f>
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B9">
-        <f>COUNTIF('Casos API'!K2:K23,"Falhou")</f>
+        <f>COUNTIF('Casos API'!L2:L23,"Falhou")</f>
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="BUGS!A2" display="UI — Falhou" xr:uid="{9BC09314-ED96-481A-8760-6B3D9F3440BC}"/>
-    <hyperlink ref="A9" location="BUGS!A3" display="API — Falhou" xr:uid="{0FB67E13-2BA2-4909-999C-275C82F4D85F}"/>
+    <hyperlink ref="A5" location="'BUG REPORT'!A2" display="UI — Falhou" xr:uid="{9BC09314-ED96-481A-8760-6B3D9F3440BC}"/>
+    <hyperlink ref="A9" location="'BUG REPORT'!A3" display="API — Falhou" xr:uid="{0FB67E13-2BA2-4909-999C-275C82F4D85F}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -8299,7 +8805,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -8315,7 +8821,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -8339,7 +8845,7 @@
         <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -8355,7 +8861,7 @@
         <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -8387,7 +8893,7 @@
         <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -8400,42 +8906,42 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -8445,92 +8951,122 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A57D3A4F-65F6-49E8-A879-CE2232515250}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="87.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="127.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="74.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="131.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="107.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C1" t="s">
+        <v>350</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>334</v>
+      </c>
+      <c r="F1" t="s">
+        <v>236</v>
+      </c>
+      <c r="G1" t="s">
         <v>335</v>
       </c>
-      <c r="B1" t="s">
+      <c r="H1" t="s">
         <v>336</v>
       </c>
-      <c r="C1" t="s">
+      <c r="I1" t="s">
         <v>337</v>
       </c>
-      <c r="D1" t="s">
-        <v>237</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="207" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B2" t="s">
         <v>338</v>
       </c>
-      <c r="F1" t="s">
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F2" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="G2" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="207" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="H2" t="s">
+        <v>341</v>
+      </c>
+      <c r="I2" t="s">
+        <v>368</v>
+      </c>
+      <c r="J2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="180.75" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>347</v>
       </c>
-      <c r="B2" t="s">
-        <v>341</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>342</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="E2" t="s">
-        <v>343</v>
-      </c>
-      <c r="F2" t="s">
-        <v>344</v>
-      </c>
-      <c r="G2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="180" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="G3" t="s">
         <v>348</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="H3" s="10" t="s">
         <v>349</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>350</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>351</v>
-      </c>
-      <c r="E3" t="s">
-        <v>352</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>353</v>
-      </c>
-      <c r="G3" t="s">
-        <v>354</v>
+      <c r="I3" t="s">
+        <v>369</v>
+      </c>
+      <c r="J3" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{43C3DF2F-69F2-4FF5-8182-6D4F43AC14FF}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{3CF88411-6D0D-40C1-B2BB-5726982DEBA1}"/>
-    <hyperlink ref="F3" r:id="rId3" display="https://app.screencast.com/nnbkJNq2WYJsT" xr:uid="{52E7D32F-0DB9-41F9-8AA8-13116EF31983}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{43C3DF2F-69F2-4FF5-8182-6D4F43AC14FF}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{3CF88411-6D0D-40C1-B2BB-5726982DEBA1}"/>
+    <hyperlink ref="H3" r:id="rId3" display="https://app.screencast.com/nnbkJNq2WYJsT" xr:uid="{52E7D32F-0DB9-41F9-8AA8-13116EF31983}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>

</xml_diff>